<commit_message>
recent best score 0.666 by simple_top5_samewrong
</commit_message>
<xml_diff>
--- a/functional_experiments.xlsx
+++ b/functional_experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Model Stealing\tml2026-team_XLIII-assignment_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207AA5AA-858D-4B9F-A469-9C94D6D641B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E686A8-33F9-40B8-9AE6-8950DB905404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="32">
   <si>
     <t>Experiment</t>
   </si>
@@ -112,6 +112,15 @@
   </si>
   <si>
     <t>single_conf_corr</t>
+  </si>
+  <si>
+    <t>target aug</t>
+  </si>
+  <si>
+    <t>simple_top5_top1</t>
+  </si>
+  <si>
+    <t>simple_top5_samewrong</t>
   </si>
 </sst>
 </file>
@@ -458,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
@@ -837,6 +846,193 @@
         <v>3</v>
       </c>
     </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>11</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>12</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>13</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>14</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>15</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>16</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>17</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>18</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>19</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>20</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>21</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0.66659999999999997</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
further top_5 weighted experiments
</commit_message>
<xml_diff>
--- a/functional_experiments.xlsx
+++ b/functional_experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Model Stealing\tml2026-team_XLIII-assignment_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 2\tml2026-team_XLIII-assignment_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E686A8-33F9-40B8-9AE6-8950DB905404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F20A6C6-669A-4F02-87E3-C8C599DF1C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="36">
   <si>
     <t>Experiment</t>
   </si>
@@ -121,6 +121,18 @@
   </si>
   <si>
     <t>simple_top5_samewrong</t>
+  </si>
+  <si>
+    <t>top5_samewrong_80_20</t>
+  </si>
+  <si>
+    <t>top5_samewrong_70_30</t>
+  </si>
+  <si>
+    <t>top5_samewrong_top1</t>
+  </si>
+  <si>
+    <t>max_top5_samewrong</t>
   </si>
 </sst>
 </file>
@@ -467,13 +479,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.140625" style="5" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.140625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1033,8 +1045,76 @@
         <v>0.66659999999999997</v>
       </c>
     </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>22</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>23</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>24</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>25</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>